<commit_message>
Done with the NSA Approval For Testing Account
</commit_message>
<xml_diff>
--- a/frontend/src/html/components/RegistrationAndPayment/Final Approval for NSA course titles_FY25 (ECSS).xlsx
+++ b/frontend/src/html/components/RegistrationAndPayment/Final Approval for NSA course titles_FY25 (ECSS).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moseslee/Desktop/ecss-cms/frontend/src/html/components/RegistrationAndPayment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C67D8B5-F19D-6A4A-A855-BEFF615F10FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327BC618-7FF6-5F4B-B19E-6E000A2CA244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28720" windowHeight="18100" xr2:uid="{A47178BE-0939-4DB7-9A02-46546E4BCF68}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
   <si>
     <t xml:space="preserve">Registered Orgn Name: </t>
   </si>
@@ -401,6 +401,15 @@
   </si>
   <si>
     <t>不和慢性病做朋友 (TCM – Don’t be a Friend of Chronic Diseases)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECSS-CBO-M-032E </t>
+  </si>
+  <si>
+    <t>(Art of Paper Quiliing)</t>
+  </si>
+  <si>
+    <t>衍纸的艺术</t>
   </si>
 </sst>
 </file>
@@ -732,22 +741,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1093,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A4B9C22-97F8-4B6E-8414-BE9E98D9A7C8}">
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -1177,56 +1186,56 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="27" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="29">
         <v>20</v>
       </c>
-      <c r="D9" s="27">
+      <c r="D9" s="31">
         <v>360</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="31">
         <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="30"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
     </row>
     <row r="11" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="27" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="29">
         <v>15</v>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="31">
         <v>250</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="31">
         <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="30"/>
+      <c r="A12" s="28"/>
       <c r="B12" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="32"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
     </row>
     <row r="13" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="17" t="s">
@@ -1246,212 +1255,212 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="27" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="29">
         <v>20</v>
       </c>
-      <c r="D14" s="27">
+      <c r="D14" s="31">
         <v>400</v>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="31">
         <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="30"/>
+      <c r="A15" s="28"/>
       <c r="B15" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="27" t="s">
         <v>23</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="29">
         <v>15</v>
       </c>
-      <c r="D16" s="27">
+      <c r="D16" s="31">
         <v>300</v>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="31">
         <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="30"/>
+      <c r="A17" s="28"/>
       <c r="B17" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="32"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="27" t="s">
         <v>26</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="29">
         <v>20</v>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="31">
         <v>360</v>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="31">
         <v>288</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="30"/>
+      <c r="A19" s="28"/>
       <c r="B19" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="27" t="s">
         <v>29</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="29">
         <v>8</v>
       </c>
-      <c r="D20" s="27">
+      <c r="D20" s="31">
         <v>200</v>
       </c>
-      <c r="E20" s="27">
+      <c r="E20" s="31">
         <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="30"/>
+      <c r="A21" s="28"/>
       <c r="B21" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
     </row>
     <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="27" t="s">
         <v>32</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="31">
+      <c r="C22" s="29">
         <v>9</v>
       </c>
-      <c r="D22" s="27">
+      <c r="D22" s="31">
         <v>254</v>
       </c>
-      <c r="E22" s="27">
+      <c r="E22" s="31">
         <v>203.2</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="30"/>
+      <c r="A23" s="28"/>
       <c r="B23" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
     </row>
     <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="27" t="s">
         <v>35</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="29">
         <v>25</v>
       </c>
-      <c r="D24" s="27">
+      <c r="D24" s="31">
         <v>460</v>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="31">
         <v>368</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="30"/>
+      <c r="A25" s="28"/>
       <c r="B25" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
     </row>
     <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="27" t="s">
         <v>38</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="29">
         <v>15</v>
       </c>
-      <c r="D26" s="27">
+      <c r="D26" s="31">
         <v>200</v>
       </c>
-      <c r="E26" s="27">
+      <c r="E26" s="31">
         <v>160</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="30"/>
+      <c r="A27" s="28"/>
       <c r="B27" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
     </row>
     <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="27" t="s">
         <v>41</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="31">
+      <c r="C28" s="29">
         <v>15</v>
       </c>
-      <c r="D28" s="27">
+      <c r="D28" s="31">
         <v>400</v>
       </c>
-      <c r="E28" s="27">
+      <c r="E28" s="31">
         <v>320</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="30"/>
+      <c r="A29" s="28"/>
       <c r="B29" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
@@ -1522,71 +1531,71 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="29" t="s">
+      <c r="A34" s="27" t="s">
         <v>51</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="31">
+      <c r="C34" s="29">
         <v>8</v>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="31">
         <v>180</v>
       </c>
-      <c r="E34" s="27">
+      <c r="E34" s="31">
         <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="30"/>
+      <c r="A35" s="28"/>
       <c r="B35" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
     </row>
     <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="27" t="s">
         <v>54</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="31">
+      <c r="C36" s="29">
         <v>16</v>
       </c>
-      <c r="D36" s="27">
+      <c r="D36" s="31">
         <v>320</v>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="31">
         <v>256</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="30"/>
+      <c r="A37" s="28"/>
       <c r="B37" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="32"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="28"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
     </row>
     <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="27" t="s">
         <v>57</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="31">
+      <c r="C38" s="29">
         <v>20</v>
       </c>
-      <c r="D38" s="27">
+      <c r="D38" s="31">
         <v>400</v>
       </c>
-      <c r="E38" s="27">
+      <c r="E38" s="31">
         <v>320</v>
       </c>
     </row>
@@ -1597,65 +1606,65 @@
       </c>
       <c r="C39" s="34"/>
       <c r="D39" s="35"/>
-      <c r="E39" s="28"/>
+      <c r="E39" s="32"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="30"/>
+      <c r="A40" s="28"/>
       <c r="B40" s="16"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="28"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="32"/>
     </row>
     <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="27" t="s">
         <v>60</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C41" s="31">
+      <c r="C41" s="29">
         <v>20</v>
       </c>
-      <c r="D41" s="27">
+      <c r="D41" s="31">
         <v>400</v>
       </c>
-      <c r="E41" s="27">
+      <c r="E41" s="31">
         <v>320</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="30"/>
+      <c r="A42" s="28"/>
       <c r="B42" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C42" s="32"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
     </row>
     <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="29" t="s">
+      <c r="A43" s="27" t="s">
         <v>63</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="31">
+      <c r="C43" s="29">
         <v>8</v>
       </c>
-      <c r="D43" s="27">
+      <c r="D43" s="31">
         <v>160</v>
       </c>
-      <c r="E43" s="27">
+      <c r="E43" s="31">
         <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="30"/>
+      <c r="A44" s="28"/>
       <c r="B44" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
     </row>
     <row r="45" spans="1:5" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="17" t="s">
@@ -1675,30 +1684,30 @@
       </c>
     </row>
     <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A46" s="29" t="s">
+      <c r="A46" s="27" t="s">
         <v>68</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C46" s="31">
+      <c r="C46" s="29">
         <v>15</v>
       </c>
-      <c r="D46" s="27">
+      <c r="D46" s="31">
         <v>200</v>
       </c>
-      <c r="E46" s="27">
+      <c r="E46" s="31">
         <v>160</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" s="30"/>
+      <c r="A47" s="28"/>
       <c r="B47" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="32"/>
     </row>
     <row r="48" spans="1:5" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
@@ -1769,56 +1778,56 @@
       </c>
     </row>
     <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="29" t="s">
+      <c r="A52" s="27" t="s">
         <v>79</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C52" s="31">
+      <c r="C52" s="29">
         <v>24</v>
       </c>
-      <c r="D52" s="27">
+      <c r="D52" s="31">
         <v>620</v>
       </c>
-      <c r="E52" s="27">
+      <c r="E52" s="31">
         <v>496</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" s="30"/>
+      <c r="A53" s="28"/>
       <c r="B53" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="C53" s="32"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="28"/>
+      <c r="C53" s="30"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
     </row>
     <row r="54" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="29" t="s">
+      <c r="A54" s="27" t="s">
         <v>82</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C54" s="31">
+      <c r="C54" s="29">
         <v>3</v>
       </c>
-      <c r="D54" s="27">
+      <c r="D54" s="31">
         <v>50</v>
       </c>
-      <c r="E54" s="27">
+      <c r="E54" s="31">
         <v>40</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="30"/>
+      <c r="A55" s="28"/>
       <c r="B55" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="C55" s="32"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="32"/>
+      <c r="E55" s="32"/>
     </row>
     <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="17" t="s">
@@ -1855,189 +1864,218 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="29" t="s">
+      <c r="A58" s="27" t="s">
         <v>89</v>
       </c>
       <c r="B58" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C58" s="31">
+      <c r="C58" s="29">
         <v>8</v>
       </c>
-      <c r="D58" s="27">
+      <c r="D58" s="31">
         <v>200</v>
       </c>
-      <c r="E58" s="27">
+      <c r="E58" s="31">
         <v>160</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="30"/>
+      <c r="A59" s="28"/>
       <c r="B59" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C59" s="32"/>
-      <c r="D59" s="28"/>
-      <c r="E59" s="28"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="32"/>
+      <c r="E59" s="32"/>
     </row>
     <row r="60" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="29" t="s">
+      <c r="A60" s="27" t="s">
         <v>92</v>
       </c>
       <c r="B60" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="C60" s="31">
+      <c r="C60" s="29">
         <v>8</v>
       </c>
-      <c r="D60" s="27">
+      <c r="D60" s="31">
         <v>160</v>
       </c>
-      <c r="E60" s="27">
+      <c r="E60" s="31">
         <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="30"/>
+      <c r="A61" s="28"/>
       <c r="B61" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="C61" s="32"/>
-      <c r="D61" s="28"/>
-      <c r="E61" s="28"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="32"/>
+      <c r="E61" s="32"/>
     </row>
     <row r="62" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A62" s="29" t="s">
+      <c r="A62" s="27" t="s">
         <v>95</v>
       </c>
       <c r="B62" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C62" s="31">
+      <c r="C62" s="29">
         <v>15</v>
       </c>
-      <c r="D62" s="27">
+      <c r="D62" s="31">
         <v>200</v>
       </c>
-      <c r="E62" s="27">
+      <c r="E62" s="31">
         <v>160</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="30"/>
+      <c r="A63" s="28"/>
       <c r="B63" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C63" s="32"/>
-      <c r="D63" s="28"/>
-      <c r="E63" s="28"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="32"/>
+      <c r="E63" s="32"/>
     </row>
     <row r="64" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="29" t="s">
+      <c r="A64" s="27" t="s">
         <v>98</v>
       </c>
       <c r="B64" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="C64" s="31">
+      <c r="C64" s="29">
         <v>15</v>
       </c>
-      <c r="D64" s="27">
+      <c r="D64" s="31">
         <v>300</v>
       </c>
-      <c r="E64" s="27">
+      <c r="E64" s="31">
         <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A65" s="30"/>
+      <c r="A65" s="28"/>
       <c r="B65" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="28"/>
-      <c r="E65" s="28"/>
+      <c r="C65" s="30"/>
+      <c r="D65" s="32"/>
+      <c r="E65" s="32"/>
     </row>
     <row r="66" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A66" s="29" t="s">
+      <c r="A66" s="27" t="s">
         <v>101</v>
       </c>
       <c r="B66" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="C66" s="31">
+      <c r="C66" s="29">
         <v>7</v>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="31">
         <v>100</v>
       </c>
-      <c r="E66" s="27">
+      <c r="E66" s="31">
         <v>80</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="30"/>
+      <c r="A67" s="28"/>
       <c r="B67" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C67" s="32"/>
-      <c r="D67" s="28"/>
-      <c r="E67" s="28"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="32"/>
+      <c r="E67" s="32"/>
     </row>
     <row r="68" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A68" s="29" t="s">
+      <c r="A68" s="27" t="s">
         <v>104</v>
       </c>
       <c r="B68" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C68" s="31">
+      <c r="C68" s="29">
         <v>16</v>
       </c>
-      <c r="D68" s="27">
+      <c r="D68" s="31">
         <v>320</v>
       </c>
-      <c r="E68" s="27">
+      <c r="E68" s="31">
         <v>256</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A69" s="30"/>
+      <c r="A69" s="28"/>
       <c r="B69" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="C69" s="32"/>
-      <c r="D69" s="28"/>
-      <c r="E69" s="28"/>
+      <c r="C69" s="30"/>
+      <c r="D69" s="32"/>
+      <c r="E69" s="32"/>
     </row>
     <row r="70" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A70" s="29" t="s">
+      <c r="A70" s="27" t="s">
         <v>107</v>
       </c>
       <c r="B70" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="C70" s="31">
+      <c r="C70" s="29">
         <v>24</v>
       </c>
-      <c r="D70" s="27">
+      <c r="D70" s="31">
         <v>500</v>
       </c>
-      <c r="E70" s="27">
+      <c r="E70" s="31">
         <v>400</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A71" s="30"/>
+      <c r="A71" s="28"/>
       <c r="B71" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C71" s="32"/>
-      <c r="D71" s="28"/>
-      <c r="E71" s="28"/>
+      <c r="C71" s="30"/>
+      <c r="D71" s="32"/>
+      <c r="E71" s="32"/>
+    </row>
+    <row r="72" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C72" s="29">
+        <v>24</v>
+      </c>
+      <c r="D72" s="31">
+        <v>180</v>
+      </c>
+      <c r="E72" s="31">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A73" s="28"/>
+      <c r="B73" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C73" s="30"/>
+      <c r="D73" s="32"/>
+      <c r="E73" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="100">
+  <mergeCells count="104">
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
     <mergeCell ref="A70:A71"/>
     <mergeCell ref="C70:C71"/>
     <mergeCell ref="D70:D71"/>
@@ -2047,81 +2085,78 @@
     <mergeCell ref="A68:A69"/>
     <mergeCell ref="C68:C69"/>
     <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
     <mergeCell ref="A58:A59"/>
     <mergeCell ref="C58:C59"/>
     <mergeCell ref="D58:D59"/>
     <mergeCell ref="A60:A61"/>
     <mergeCell ref="C60:C61"/>
     <mergeCell ref="D60:D61"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
     <mergeCell ref="A52:A53"/>
     <mergeCell ref="C52:C53"/>
     <mergeCell ref="D52:D53"/>
     <mergeCell ref="A54:A55"/>
     <mergeCell ref="C54:C55"/>
     <mergeCell ref="D54:D55"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
     <mergeCell ref="A38:A40"/>
     <mergeCell ref="C38:C40"/>
     <mergeCell ref="D38:D40"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="C41:C42"/>
     <mergeCell ref="D41:D42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="C34:C35"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="C36:C37"/>
     <mergeCell ref="D36:D37"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="C22:C23"/>
     <mergeCell ref="D22:D23"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="D24:D25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="D18:D19"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="D20:D21"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A72:A73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="E72:E73"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="E64:E65"/>
     <mergeCell ref="E66:E67"/>
@@ -2138,6 +2173,10 @@
     <mergeCell ref="E58:E59"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E34:E35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>

</xml_diff>